<commit_message>
fix excel BBSL STDSX
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/BM_TongHopSanLuong - KCS.xlsx
+++ b/dataproduct.api/wwwroot/templates/BM_TongHopSanLuong - KCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\03. ThongKePKH\DATAPRODUCT_V2\dataproduct.api\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8985D79-2932-4FD1-A5E9-4AC46BBE10AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EADA18-F280-4A3F-AB1E-A8CC538C46DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{77908C05-ABC3-4C3F-A6F5-1B05425144FB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>STT</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>KL Cân</t>
+  </si>
+  <si>
+    <t>Phân loại</t>
   </si>
 </sst>
 </file>
@@ -277,6 +280,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -315,24 +336,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -692,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43BAB014-E6DF-4BFD-BF20-A00AB0E3B9F2}">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="1" customWidth="1"/>
@@ -705,143 +708,150 @@
     <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="17" style="1" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="39.85546875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="24.5703125" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="1"/>
+    <col min="11" max="12" width="19" style="1" customWidth="1"/>
+    <col min="13" max="13" width="16.85546875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="39.85546875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="24.5703125" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22"/>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+    <row r="1" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="13"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="2" spans="1:14" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
+    <row r="2" spans="1:15" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+    <row r="3" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
     </row>
-    <row r="4" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
     </row>
-    <row r="5" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="18" t="s">
+      <c r="J6" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="21" t="s">
+      <c r="K6" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="L6" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="M6" s="12" t="s">
+      <c r="N6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="O6" s="15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="10"/>
+    <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="16"/>
     </row>
-    <row r="8" spans="1:14" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="11"/>
+    <row r="8" spans="1:15" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="17"/>
     </row>
-    <row r="9" spans="1:14" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="5"/>
@@ -853,19 +863,20 @@
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="6"/>
+      <c r="M9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="6"/>
-      <c r="N9" s="7"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="7"/>
     </row>
-    <row r="10" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:14" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:15" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -882,24 +893,25 @@
     <row r="30" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A4:N4"/>
+  <mergeCells count="18">
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:D8"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A4:O4"/>
+    <mergeCell ref="O6:O8"/>
     <mergeCell ref="N6:N8"/>
     <mergeCell ref="M6:M8"/>
-    <mergeCell ref="L6:L8"/>
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="I6:I8"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="K6:K8"/>
+    <mergeCell ref="L6:L8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -916,15 +928,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076634EE74CE1ED46AEEF0EBAEBE54F1E" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b3c6bda8a7649ee342e145cf9ea6f2d9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7bdf782f-2886-4011-99ee-a2495b2dfaf9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c0379f6dc3a2273300603944198f78b4" ns3:_="">
     <xsd:import namespace="7bdf782f-2886-4011-99ee-a2495b2dfaf9"/>
@@ -1100,6 +1103,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{847D81C1-0646-4BD0-BC63-D9DF50568213}">
   <ds:schemaRefs>
@@ -1117,14 +1129,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24B1C2B3-91A9-494D-BEB6-2B1BB33BE342}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CEB506B-C232-407B-9B3B-8F4E72E7BB4D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1140,4 +1144,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24B1C2B3-91A9-494D-BEB6-2B1BB33BE342}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>